<commit_message>
refactor(services): improve date parsing robustness
Update `excel_reader.py` to better handle `pd.Timestamp` and additional null-like strings ('<NA>', 'NaT'). Removed unused imports and cleaned up `mapping.py` to improve maintainability.
</commit_message>
<xml_diff>
--- a/output/HSE_Action_Tracking_Register_JSL.xlsx
+++ b/output/HSE_Action_Tracking_Register_JSL.xlsx
@@ -717,7 +717,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA15"/>
+  <dimension ref="A1:AA16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -770,7 +770,7 @@
         </is>
       </c>
       <c r="AA3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
@@ -781,7 +781,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>18-Sep-26</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr">
@@ -802,7 +802,7 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
@@ -832,7 +832,7 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11" ht="26" customHeight="1">
@@ -913,7 +913,7 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>HSCO-OR-01</t>
+          <t>HSCO-OB-01</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
@@ -923,27 +923,23 @@
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>15-Sep-26</t>
-        </is>
-      </c>
-      <c r="E12" s="9" t="inlineStr">
-        <is>
-          <t>Substation 1</t>
-        </is>
-      </c>
+          <t>01/09/2026</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr"/>
       <c r="F12" s="10" t="inlineStr">
         <is>
-          <t>Damaged electrical cable</t>
+          <t>Obs 1</t>
         </is>
       </c>
       <c r="G12" s="10" t="inlineStr">
         <is>
-          <t>Replace cable immediately</t>
+          <t>Rec 1</t>
         </is>
       </c>
       <c r="H12" s="9" t="inlineStr">
         <is>
-          <t>Officer Mike</t>
+          <t>Safety A</t>
         </is>
       </c>
       <c r="I12" s="9" t="inlineStr">
@@ -956,11 +952,7 @@
           <t>HEISCO</t>
         </is>
       </c>
-      <c r="K12" s="9" t="inlineStr">
-        <is>
-          <t>15-Sep-26</t>
-        </is>
-      </c>
+      <c r="K12" s="9" t="inlineStr"/>
       <c r="L12" s="9" t="inlineStr">
         <is>
           <t>General</t>
@@ -979,7 +971,7 @@
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>HSCO-OR-02</t>
+          <t>HSCO-OB-02</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
@@ -989,27 +981,23 @@
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>16-Sep-26</t>
-        </is>
-      </c>
-      <c r="E13" s="9" t="inlineStr">
-        <is>
-          <t>Storage Yard</t>
-        </is>
-      </c>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr"/>
       <c r="F13" s="10" t="inlineStr">
         <is>
-          <t>Missing fire extinguisher tag</t>
+          <t>Obs 2</t>
         </is>
       </c>
       <c r="G13" s="10" t="inlineStr">
         <is>
-          <t>Inspect and tag extinguisher</t>
+          <t>Rec 2</t>
         </is>
       </c>
       <c r="H13" s="9" t="inlineStr">
         <is>
-          <t>Officer Sarah</t>
+          <t>Safety A</t>
         </is>
       </c>
       <c r="I13" s="9" t="inlineStr">
@@ -1022,11 +1010,7 @@
           <t>HEISCO</t>
         </is>
       </c>
-      <c r="K13" s="9" t="inlineStr">
-        <is>
-          <t>16-Sep-26</t>
-        </is>
-      </c>
+      <c r="K13" s="9" t="inlineStr"/>
       <c r="L13" s="9" t="inlineStr">
         <is>
           <t>General</t>
@@ -1045,7 +1029,7 @@
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>HSCO-OR-03</t>
+          <t>HSCO-OB-03</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
@@ -1055,27 +1039,23 @@
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>17-Sep-26</t>
-        </is>
-      </c>
-      <c r="E14" s="9" t="inlineStr">
-        <is>
-          <t>Pump House</t>
-        </is>
-      </c>
+          <t>03/09/2026</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr"/>
       <c r="F14" s="10" t="inlineStr">
         <is>
-          <t>Uncovered trench</t>
+          <t>Obs 3</t>
         </is>
       </c>
       <c r="G14" s="10" t="inlineStr">
         <is>
-          <t>Install barricade and cover</t>
+          <t>Rec 3</t>
         </is>
       </c>
       <c r="H14" s="9" t="inlineStr">
         <is>
-          <t>Officer Mike</t>
+          <t>Safety A</t>
         </is>
       </c>
       <c r="I14" s="9" t="inlineStr">
@@ -1088,11 +1068,7 @@
           <t>HEISCO</t>
         </is>
       </c>
-      <c r="K14" s="9" t="inlineStr">
-        <is>
-          <t>17-Sep-26</t>
-        </is>
-      </c>
+      <c r="K14" s="9" t="inlineStr"/>
       <c r="L14" s="9" t="inlineStr">
         <is>
           <t>General</t>
@@ -1111,7 +1087,7 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>HSCO-OR-04</t>
+          <t>HSCO-OB-04</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
@@ -1121,27 +1097,23 @@
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>18-Sep-26</t>
-        </is>
-      </c>
-      <c r="E15" s="9" t="inlineStr">
-        <is>
-          <t>Gate 2</t>
-        </is>
-      </c>
+          <t>04/09/2026</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr"/>
       <c r="F15" s="10" t="inlineStr">
         <is>
-          <t>No safety helmet</t>
+          <t>Obs 4</t>
         </is>
       </c>
       <c r="G15" s="10" t="inlineStr">
         <is>
-          <t>Provide PPE</t>
+          <t>Rec 4</t>
         </is>
       </c>
       <c r="H15" s="9" t="inlineStr">
         <is>
-          <t>Officer Sarah</t>
+          <t>Safety A</t>
         </is>
       </c>
       <c r="I15" s="9" t="inlineStr">
@@ -1154,11 +1126,7 @@
           <t>HEISCO</t>
         </is>
       </c>
-      <c r="K15" s="9" t="inlineStr">
-        <is>
-          <t>18-Sep-26</t>
-        </is>
-      </c>
+      <c r="K15" s="9" t="inlineStr"/>
       <c r="L15" s="9" t="inlineStr">
         <is>
           <t>General</t>
@@ -1170,6 +1138,64 @@
         </is>
       </c>
       <c r="N15" s="10" t="inlineStr"/>
+    </row>
+    <row r="16" ht="32" customHeight="1">
+      <c r="A16" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>HSCO-OB-05</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Site Observation</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>05/09/2026</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr"/>
+      <c r="F16" s="10" t="inlineStr">
+        <is>
+          <t>Obs 5</t>
+        </is>
+      </c>
+      <c r="G16" s="10" t="inlineStr">
+        <is>
+          <t>Rec 5</t>
+        </is>
+      </c>
+      <c r="H16" s="9" t="inlineStr">
+        <is>
+          <t>Safety A</t>
+        </is>
+      </c>
+      <c r="I16" s="9" t="inlineStr">
+        <is>
+          <t>Unsafe Condition</t>
+        </is>
+      </c>
+      <c r="J16" s="9" t="inlineStr">
+        <is>
+          <t>HEISCO</t>
+        </is>
+      </c>
+      <c r="K16" s="9" t="inlineStr"/>
+      <c r="L16" s="9" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="M16" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N16" s="10" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
chore: update sample observation data
Refreshed session data and output files with new observation entries for testing purposes.
</commit_message>
<xml_diff>
--- a/output/HSE_Action_Tracking_Register_JSL.xlsx
+++ b/output/HSE_Action_Tracking_Register_JSL.xlsx
@@ -717,7 +717,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA16"/>
+  <dimension ref="A1:AA15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -770,7 +770,7 @@
         </is>
       </c>
       <c r="AA3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
@@ -781,7 +781,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>05/09/2026</t>
+          <t>13/09/2026</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr">
@@ -802,7 +802,7 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
@@ -832,7 +832,7 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11" ht="26" customHeight="1">
@@ -923,23 +923,23 @@
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>01/09/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr"/>
       <c r="F12" s="10" t="inlineStr">
         <is>
-          <t>Obs 1</t>
+          <t>Finding A</t>
         </is>
       </c>
       <c r="G12" s="10" t="inlineStr">
         <is>
-          <t>Rec 1</t>
+          <t>Action A</t>
         </is>
       </c>
       <c r="H12" s="9" t="inlineStr">
         <is>
-          <t>Safety A</t>
+          <t>Officer 1</t>
         </is>
       </c>
       <c r="I12" s="9" t="inlineStr">
@@ -981,23 +981,23 @@
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>02/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr"/>
       <c r="F13" s="10" t="inlineStr">
         <is>
-          <t>Obs 2</t>
+          <t>Finding B</t>
         </is>
       </c>
       <c r="G13" s="10" t="inlineStr">
         <is>
-          <t>Rec 2</t>
+          <t>Action B</t>
         </is>
       </c>
       <c r="H13" s="9" t="inlineStr">
         <is>
-          <t>Safety A</t>
+          <t>Officer 1</t>
         </is>
       </c>
       <c r="I13" s="9" t="inlineStr">
@@ -1039,23 +1039,23 @@
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>03/09/2026</t>
+          <t>12/09/2026</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr"/>
       <c r="F14" s="10" t="inlineStr">
         <is>
-          <t>Obs 3</t>
+          <t>Finding C</t>
         </is>
       </c>
       <c r="G14" s="10" t="inlineStr">
         <is>
-          <t>Rec 3</t>
+          <t>Action C</t>
         </is>
       </c>
       <c r="H14" s="9" t="inlineStr">
         <is>
-          <t>Safety A</t>
+          <t>Officer 1</t>
         </is>
       </c>
       <c r="I14" s="9" t="inlineStr">
@@ -1097,23 +1097,23 @@
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>04/09/2026</t>
+          <t>13/09/2026</t>
         </is>
       </c>
       <c r="E15" s="9" t="inlineStr"/>
       <c r="F15" s="10" t="inlineStr">
         <is>
-          <t>Obs 4</t>
+          <t>Finding D</t>
         </is>
       </c>
       <c r="G15" s="10" t="inlineStr">
         <is>
-          <t>Rec 4</t>
+          <t>Action D</t>
         </is>
       </c>
       <c r="H15" s="9" t="inlineStr">
         <is>
-          <t>Safety A</t>
+          <t>Officer 1</t>
         </is>
       </c>
       <c r="I15" s="9" t="inlineStr">
@@ -1138,64 +1138,6 @@
         </is>
       </c>
       <c r="N15" s="10" t="inlineStr"/>
-    </row>
-    <row r="16" ht="32" customHeight="1">
-      <c r="A16" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>HSCO-OB-05</t>
-        </is>
-      </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t>Site Observation</t>
-        </is>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t>05/09/2026</t>
-        </is>
-      </c>
-      <c r="E16" s="9" t="inlineStr"/>
-      <c r="F16" s="10" t="inlineStr">
-        <is>
-          <t>Obs 5</t>
-        </is>
-      </c>
-      <c r="G16" s="10" t="inlineStr">
-        <is>
-          <t>Rec 5</t>
-        </is>
-      </c>
-      <c r="H16" s="9" t="inlineStr">
-        <is>
-          <t>Safety A</t>
-        </is>
-      </c>
-      <c r="I16" s="9" t="inlineStr">
-        <is>
-          <t>Unsafe Condition</t>
-        </is>
-      </c>
-      <c r="J16" s="9" t="inlineStr">
-        <is>
-          <t>HEISCO</t>
-        </is>
-      </c>
-      <c r="K16" s="9" t="inlineStr"/>
-      <c r="L16" s="9" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="M16" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="N16" s="10" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>